<commit_message>
Move lamps, flashlights, tablets, Trodat, pen holders to Ruziboev Sindor
</commit_message>
<xml_diff>
--- a/groups.xlsx
+++ b/groups.xlsx
@@ -436,7 +436,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Равшанов Зиёдулло</t>
+          <t>Рузибоев Синдор</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Равшанов Зиёдулло</t>
+          <t>Рузибоев Синдор</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Мустафоев Абдулло</t>
+          <t>Рузибоев Синдор</t>
         </is>
       </c>
     </row>
@@ -1648,7 +1648,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Мустафоев Абдулло</t>
+          <t>Рузибоев Синдор</t>
         </is>
       </c>
     </row>
@@ -1660,7 +1660,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Равшанов Зиёдулло</t>
+          <t>Рузибоев Синдор</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Мустафоев Абдулло</t>
+          <t>Рузибоев Синдор</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Тохиров Муслимбек</t>
+          <t>Рузибоев Синдор</t>
         </is>
       </c>
     </row>
@@ -2332,7 +2332,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Тохиров Муслимбек</t>
+          <t>Рузибоев Синдор</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Move inks and paints folders to Toxirov Muslimbek
</commit_message>
<xml_diff>
--- a/groups.xlsx
+++ b/groups.xlsx
@@ -472,7 +472,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Равшанов Зиёдулло</t>
+          <t>Тохиров Муслимбек</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Равшанов Зиёдулло</t>
+          <t>Тохиров Муслимбек</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Ядуллаев Умид</t>
+          <t>Тохиров Муслимбек</t>
         </is>
       </c>
     </row>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Ядуллаев Умид</t>
+          <t>Тохиров Муслимбек</t>
         </is>
       </c>
     </row>
@@ -1792,7 +1792,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Тувалов Фаррух</t>
+          <t>Тохиров Муслимбек</t>
         </is>
       </c>
     </row>
@@ -2200,7 +2200,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Тувалов Фаррух</t>
+          <t>Тохиров Муслимбек</t>
         </is>
       </c>
     </row>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Ядуллаев Умид</t>
+          <t>Тохиров Муслимбек</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Return gouache and watercolor to Ravshanov; ink and coloring books to Farrux
</commit_message>
<xml_diff>
--- a/groups.xlsx
+++ b/groups.xlsx
@@ -472,7 +472,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Тохиров Муслимбек</t>
+          <t>Равшанов Зиёдулло</t>
         </is>
       </c>
     </row>
@@ -748,7 +748,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Тохиров Муслимбек</t>
+          <t>Равшанов Зиёдулло</t>
         </is>
       </c>
     </row>
@@ -1792,7 +1792,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Тохиров Муслимбек</t>
+          <t>Тувалов Фаррух</t>
         </is>
       </c>
     </row>
@@ -2200,7 +2200,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Тохиров Муслимбек</t>
+          <t>Тувалов Фаррух</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: Umid papkalari Ergashev Ozodbek ga biriktirildi (Excel + migratsiya)
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/groups.xlsx
+++ b/groups.xlsx
@@ -1024,7 +1024,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Ядуллаев Умид</t>
+          <t>Ergashev Ozodbek</t>
         </is>
       </c>
     </row>
@@ -1084,7 +1084,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Ядуллаев Умид</t>
+          <t>Ergashev Ozodbek</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Ядуллаев Умид</t>
+          <t>Ergashev Ozodbek</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Ядуллаев Умид</t>
+          <t>Ergashev Ozodbek</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Ядуллаев Умид</t>
+          <t>Ergashev Ozodbek</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1528,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Ядуллаев Умид</t>
+          <t>Ergashev Ozodbek</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Ядуллаев Умид</t>
+          <t>Ergashev Ozodbek</t>
         </is>
       </c>
     </row>
@@ -1924,7 +1924,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Ядуллаев Умид</t>
+          <t>Ergashev Ozodbek</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1948,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Ядуллаев Умид</t>
+          <t>Ergashev Ozodbek</t>
         </is>
       </c>
     </row>
@@ -1960,7 +1960,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Ядуллаев Умид</t>
+          <t>Ergashev Ozodbek</t>
         </is>
       </c>
     </row>
@@ -1972,7 +1972,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Ядуллаев Умид</t>
+          <t>Ergashev Ozodbek</t>
         </is>
       </c>
     </row>
@@ -2380,7 +2380,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Ядуллаев Умид</t>
+          <t>Ergashev Ozodbek</t>
         </is>
       </c>
     </row>
@@ -2392,7 +2392,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Ядуллаев Умид</t>
+          <t>Ergashev Ozodbek</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Ядуллаев Умид</t>
+          <t>Ergashev Ozodbek</t>
         </is>
       </c>
     </row>
@@ -2428,7 +2428,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Ядуллаев Умид</t>
+          <t>Ergashev Ozodbek</t>
         </is>
       </c>
     </row>
@@ -2464,7 +2464,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Ядуллаев Умид</t>
+          <t>Ergashev Ozodbek</t>
         </is>
       </c>
     </row>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Ядуллаев Умид</t>
+          <t>Ergashev Ozodbek</t>
         </is>
       </c>
     </row>

</xml_diff>